<commit_message>
Golden Path Block: full re-run on v109.24, 3 new cases (ton variance, QC Note, credit note), green 'changed this round' flags
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-block-purchase-to-cut.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-block-purchase-to-cut.xlsx
@@ -487,14 +487,14 @@
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 11</t>
+          <t>Total test cases: 14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 10 / 1 / 0</t>
+          <t>High / Medium / Low: 11 / 3 / 0</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -710,7 +710,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>PO ขึ้นสถานะ Purchase Order — Quantity 14.00 ลบ.ม., Price / Ton 10,000.00, ยอดก่อน VAT 378,000.00 บาท และมีปุ่มสมาร์ท Receipt 1 ใบ (ตัวอย่างจริง P00086)</t>
+          <t>PO ขึ้นสถานะ Purchase Order — Quantity 14.00 ลบ.ม., Price / Ton 10,000.00, ยอดก่อน VAT 378,000.00 บาท และมีปุ่มสมาร์ท Receipt 1 ใบ (ตัวอย่างจริง P00295)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>ช่อง "จำนวน" บน PO คือปริมาณโดยประมาณที่สั่ง ไม่ใช่จำนวนก้อน ขนาดจริงของแต่ละก้อนจะกรอกตอนรับของ · ✅ ตัวเลขตันที่หาร 2.7 ไม่ลงตัว (เช่น 10 ตัน) เคยแสดงเพี้ยนเป็น 9.99 ตัน แก้แล้ว (11 ต.ค. 2569) แต่ยอดเงินอาจต่างประมาณ 0.10 บาท จึงใช้ตันที่หาร 2.7 ลงตัวในตัวอย่าง</t>
+          <t>ช่อง "จำนวน" บน PO คือปริมาณโดยประมาณที่สั่ง ไม่ใช่จำนวนก้อน ขนาดจริงของแต่ละก้อนจะกรอกตอนรับของ</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -742,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -762,7 +762,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>B. รับ Block เข้าคลัง (Receipt) — 1 แถว = 1 ก้อนจริง กรอกขนาดแล้ว Validate ระบบสร้างเอกสาร Block ให้เอง</t>
+          <t>B. รับ Block เข้าคลัง (Receipt) — 1 แถว = 1 ก้อนจริง กรอกขนาดและตันตามใบส่งของ แล้ว Validate ระบบสร้างเอกสาร Block ให้เอง</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>รับ Block 2 ก้อน กรอกขนาดรายก้อน แล้ว Validate</t>
+          <t>รับ Block 2 ก้อน กรอกขนาดและตันตามใบส่งของรายก้อน แล้ว Validate</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -848,20 +848,20 @@
         <is>
           <t>1. ที่ PO กดปุ่ม Receipt เพื่อเปิดใบรับของ
 2. กดคำว่า Details ที่แถว Block
-3. แถวแรกกรอก ยาว / กว้าง / สูง แล้วกด Add a line เพิ่มแถวที่สอง กรอกขนาดก้อนที่สอง
+3. แถวแรกกรอก ยาว / กว้าง / สูง และ ตันตามใบส่งของ แล้วกด Add a line เพิ่มแถวที่สอง กรอกก้อนที่สอง
 4. กด Save แล้วกด Validate
 5. เมื่อถาม Backorder เลือก No Backorder</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>ก้อนที่ 1 = 2.90 × 1.60 × 1.50 ม.
-ก้อนที่ 2 = 2.75 × 1.55 × 1.45 ม.</t>
+          <t>ก้อนที่ 1 = 2.90 × 1.60 × 1.50 ม. · 18.800 ตัน
+ก้อนที่ 2 = 2.75 × 1.55 × 1.45 ม. · 16.700 ตัน</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบรับของเป็น Done — ปลายทาง Stone Inventory/Stone Available, Quantity 13.14 ลบ.ม. (6.96 + 6.18), Qty (Ton) 35.48 ระบบสร้าง Block 2 เอกสาร: BLK-26-0029 (6.96 ลบ.ม.) และ BLK-26-0030 (6.18 ลบ.ม.)</t>
+          <t>ใบรับของเป็น Done — ปลายทาง Stone Inventory/Stone Available, Quantity 13.14 ลบ.ม. (6.96 + 6.18) ระบบสร้าง Block 2 เอกสาร: BLK-26-0385 (6.96 ลบ.ม. · 18.80 ตัน) และ BLK-26-0386 (6.18 ลบ.ม. · 16.70 ตัน) รวม 35.50 ตัน (ตัวอย่างจริง EG01/IN/00360) · ไม่มี error ตอนกด No Backorder</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -871,7 +871,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>รับน้อยกว่าที่สั่ง (13.14 จาก 14.00) ระบบถามเรื่อง Backorder ให้เลือก No Backorder เพราะผู้ขายส่งครบแล้ว · หลัง Validate มีข้อความมุมจอทีละก้อน (ปิดด้วยปุ่ม x ได้)</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — เพิ่มช่อง "ตันตามใบส่งของ" และช่อง QC Note ในหน้า Details · ตันที่กรอกกลายเป็นตันของ Block ก้อนนั้น (ใช้คิดมูลค่าสต็อกและบิลผู้ขาย) · แก้บั๊ก: เคยกด No Backorder แล้วระบบฟ้อง "กรุณากรอก ยาว × กว้าง × สูง" ตอนนี้ผ่านปกติ
+รับน้อยกว่าที่สั่ง (13.14 จาก 14.00) ระบบถามเรื่อง Backorder ให้เลือก No Backorder เพราะผู้ขายส่งครบแล้ว · ใบรับของถูกแยกเป็น 2 แถว (1 แถวต่อก้อน) แถวแรก Demand 7.82 Quantity 6.96 แถวที่สอง 6.18 / 6.18 รวมเท่า Demand เดิม 14.00 · หลัง Validate มีข้อความมุมจอทีละก้อน (ปิดด้วยปุ่ม x ได้) · ช่องตันตามใบส่งของเว้นว่างได้ ระบบจะใช้ ลบ.ม. × 2.7 แทน</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -882,34 +883,37 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-GP-BPC-03</t>
+          <t>TC-GP-BPC-12</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>ดู Block ที่เพิ่งรับเข้าคลัง</t>
+          <t>ตันตามใบส่งของไม่ตรงกับ CBM ที่วัด (เกิน 5%) — ระบบเตือนและบันทึก QC Note</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-BPC-02 เสร็จแล้ว</t>
+          <t>ทำ TC-GP-BPC-01 เสร็จแล้ว (ใช้ PO แยกอีกใบ ไม่ใช่ใบเดียวกับ BPC-02)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดแอป Stone Slab &gt; Blocks
-2. ค้นหา BLK-26-0029 เปิดดูรายละเอียด
-3. ดูการ์ดสรุปด้านบนและลองคลิกแท็บต่างๆ</t>
+          <t>1. ที่ PO ใบใหม่กด Receipt แล้วกด Details
+2. กรอกขนาดก้อนและ ตันตามใบส่งของ ที่ต่างจาก CBM × 2.7 เกิน 5%
+3. กด Save แล้วกด Validate
+4. ดูแถบเหลืองด้านบนใบรับของ แล้วเปิด Block ที่เพิ่งสร้าง</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PO = 1.00 ลบ.ม.
+Block = 1.00 × 1.00 × 1.00 ม. (CBM × 2.7 = 2.70 ตัน)
+ตันตามใบส่งของ = 3.000 ตัน (+11%)</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>การ์ดสรุปแสดง ขนาดก้อน 2.90 × 1.60 × 1.50 = 6.96 CBM · 18.79 ตัน, คงเหลือ 6.96 CBM, ราคาขายเป็นบาท/ตัน, ผลการตัด "ยังไม่ได้ตัด" พร้อมจำนวนแผ่นโดยประมาณ, ต้นทุน 10,000 บาท/ตัน และเลข PO (P00086) ช่องขนาดเป็นสีเทา แก้ตรงๆ ไม่ได้</t>
+          <t>ใบรับของ Done แถบเหลือง 2 แถบ: "ตันตามใบส่งของไม่ตรงกับ CBM ที่วัด (เกิน 5%) — ตรวจขนาดก้อนหรือใบส่งของ" และ "มี QC Note" · Block ที่สร้าง (ตัวอย่างจริง BLK-26-0388) มี QC Note บันทึกข้อความเตือนไว้ (ตัวอย่างจริง P00297 → EG01/IN/00362)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -917,11 +921,114 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="7" t="n"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ฟีเจอร์ใหม่จากการประชุม 12 ต.ค. (QC Note บนใบรับของ + เตือนตันคลาด ±5%)
+ระบบไม่ขวางการรับของ แค่ขึ้นแถบเหลืองบนใบรับของและเขียนข้อความลง QC Note ของ Block ให้ ฝ่ายคลังตามไปตรวจขนาดก้อนหรือใบส่งของได้ทีหลัง · แสดงทั้งที่ใบรับของ, PO และหน้า Block (ตัวกรอง "มี QC Note")</t>
+        </is>
+      </c>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
       <c r="L5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-BPC-03</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>ดู Block ที่เพิ่งรับเข้าคลัง</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-BPC-02 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดแอป Stone Slab &gt; Blocks
+2. ค้นหา BLK-26-0385 เปิดดูรายละเอียด
+3. ดูการ์ดสรุปด้านบนและลองคลิกแท็บต่างๆ</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>การ์ดสรุปแสดง ขนาดก้อน 2.90 × 1.60 × 1.50 = 6.96 CBM · 18.80 ตัน, คงเหลือ 6.96 CBM, ราคาขาย 26,000 บาท/ตัน (70,200 บาท/CBM), ผลการตัด "ยังไม่ได้ตัด" ประมาณ 72 แผ่น / 348.00 ตร.ม., ต้นทุน 10,000 บาท/ตัน (27,000 บาท/CBM) และเลข PO (P00295) · ด้านบนมี % สูญเสียที่ใช้ 15.00 (ค่าเริ่มต้นของบริษัท) · ช่องขนาดเป็นสีเทา แก้ตรงๆ ไม่ได้</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — การ์ดสรุปใช้ตันตามใบส่งของ (18.80 ไม่ใช่ 18.79) · มีส่วน "% สูญเสียจากการเลื่อย" และช่อง QC Note ด้านบน · จำนวนแผ่นโดยประมาณหักสูญเสียเลื่อยแล้ว
+</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-BPC-13</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>เพิ่มหรือแก้ QC Note ของ Block หลังรับของแล้ว</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-BPC-02 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิด Stone Slab &gt; Blocks &gt; BLK-26-0386
+2. ช่อง QC Note ด้านบนพิมพ์หมายเหตุ
+3. กด Save</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>QC Note = มีรอยร้าวเส้นผมด้านข้าง 1 จุด สีเข้มกว่าก้อนอื่นเล็กน้อย</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>หน้า Block ขึ้นแถบเหลือง "มี QC Note — แก้ล่าสุดโดย Administrator เมื่อ …" และข้อความที่พิมพ์แสดงในช่อง QC Note</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ฟีเจอร์ใหม่จากการประชุม 12 ต.ค.
+QC Note แก้ได้ตลอดแม้ใบรับของ Done แล้ว · ระบบเก็บชื่อผู้แก้และเวลาให้ และขึ้นแถบเหลือง "มี QC Note" บนหน้า Block</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -957,7 +1064,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>C. เก็บเงิน (Vendor Bill) — บิลผู้ขายคิดตามที่รับจริง ไม่ใช่ตามที่สั่ง</t>
+          <t>C. เก็บเงิน (Vendor Bill) — บิลผู้ขายเป็นหน่วยตัน ตามตันที่รับจริง ไม่ใช่ตามที่สั่ง</t>
         </is>
       </c>
     </row>
@@ -1043,18 +1150,18 @@
         <is>
           <t>1. เปิดแอป Accounting &gt; Vendors &gt; Bills &gt; New
 2. เลือก Vendor ที่ช่อง Auto-Complete เลือกใบสั่งซื้อ
-3. ตรวจรายการที่ระบบดึงมา แล้วกด Confirm</t>
+3. กรอก Bill Date ตรวจรายการที่ระบบดึงมา แล้วกด Confirm</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Vendor = A-Test-Vender
-Auto-Complete = P00086</t>
+Auto-Complete = P00295</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัด Block: Qty (Ton) 35.48 · Quantity 13.14 ลบ.ม. · Price 27,000.00 · Price / Ton 10,000.00 · Amount 354,780.00 บาท ท้ายบิล VAT 7% 24,834.60, Total 379,614.60 บาท สถานะ Posted และมีปุ่ม Purchases P00086 ที่หัวบิล (ตัวอย่างจริง BILL/2026/10/0003)</t>
+          <t>บรรทัด Block: Qty (Ton) 35.50 · Quantity 35.500 หน่วย ตัน (2.7 ตัน/ลบ.ม.) · Price 10,000.00 · Price / Ton 10,000.00 · Amount 355,000.00 บาท ท้ายบิล VAT 7% 24,850.00, Total 379,850.00 บาท สถานะ Posted และมีปุ่ม Purchases P00295 ที่หัวบิล (ตัวอย่างจริง BILL/2026/10/0006)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1064,7 +1171,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>บิลดึงปริมาณตามที่รับจริง (13.14) ไม่ใช่ที่สั่ง (14.00) · บรรทัดบิลแสดง Qty (Ton) หน้า Quantity และ Price / Ton หลัง Price (เพิ่ม 11 ต.ค. 2569)</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — บิลผู้ขายของ Block เป็น "ตัน" (หน่วย ตัน (2.7 ตัน/ลบ.ม.)) = ตันตามใบส่งของ × ราคาต่อตัน แทนที่จะเป็น ลบ.ม. × ราคาต่อ ลบ.ม. เดิม · ปริมาณแสดง 3 ตำแหน่ง · แก้บั๊ก: บรรทัดบิลเคยแสดง Qty (Ton) และ Price / Ton เพี้ยน (เช่น 27.81 และ 3,703.70) เพราะแปลงหน่วยซ้ำ
+บิลดึงตันที่รับจริง (35.500) ไม่ใช่ที่สั่ง (37.800) · ต้องกรอก Bill Date ก่อน Confirm (ช่องแดงถ้ายังว่าง) · ยอดเงินต่างจากคิดตาม ลบ.ม. เดิมเล็กน้อย (355,000 แทน 354,780) เพราะตันตามใบส่งของ 35.50 ต่างจากตันที่คำนวณจาก CBM 35.478</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1190,7 +1298,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Stone Slab &gt; Blocks &gt; BLK-26-0029
+          <t>1. เปิด Stone Slab &gt; Blocks &gt; BLK-26-0385
 2. กดปุ่ม แก้ขนาด (มุมซ้ายบน)
 3. ช่อง สูงใหม่ (ม.) กรอกค่าใหม่ ช่องเหตุผลที่แก้ไข กรอกเหตุผล
 4. กดปุ่ม แก้ขนาด ในหน้าต่าง</t>
@@ -1204,7 +1312,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>การ์ดสรุปเปลี่ยนเป็น 2.90 × 1.60 × 1.45 = 6.73 CBM · 18.17 ตัน คงเหลือ 6.73 CBM และมีแท็บ ประวัติแก้ขนาด (แท็บสุดท้าย) 1 แถว: สูง 1.500 → 1.450, ปริมาตร 6.96 → 6.73, ปรับสต็อก -0.23, เหตุผล และชื่อผู้แก้</t>
+          <t>การ์ดสรุปเปลี่ยนเป็น 2.90 × 1.60 × 1.45 = 6.73 CBM · 18.80 ตัน คงเหลือ 6.73 CBM (ประมาณ 70 แผ่น / 336.40 ตร.ม.) และมีแท็บ ประวัติแก้ขนาด (แท็บสุดท้าย) 1 แถว: สูง 1.500 → 1.450, ปริมาตร 6.9600 → 6.7280, ปรับสต็อก -0.23, เหตุผล และชื่อผู้แก้</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1214,7 +1322,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>บิลผู้ขายที่ Posted ไปแล้วไม่เปลี่ยน (ยังเป็น 13.14) เพราะคิดจากที่รับตอนรับของ</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ตันตามใบส่งของของ Block ไม่เปลี่ยนตามขนาดใหม่ (ยังเป็น 18.80) · ผลการตัดโดยประมาณปรับตามขนาดใหม่และหักสูญเสียเลื่อย
+บิลผู้ขายที่ Posted ไปแล้วไม่เปลี่ยน (ยังเป็น 35.500 ตัน) เพราะคิดจากที่รับตอนรับของ</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1335,7 +1444,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-BPC-02 เสร็จแล้ว (ใช้ BLK-26-0030 ซึ่งยังไม่เคยตัด)</t>
+          <t>ทำ TC-GP-BPC-02 เสร็จแล้ว (ใช้ BLK-26-0386 ซึ่งยังไม่เคยตัด)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1349,7 +1458,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Block = BLK-26-0030
+          <t>Block = BLK-26-0386
 ขนาดแผ่น = 2.75 × 1.45 ม.
 Finish = Polished · ความหนา = 2 cm
 เหตุผล = งานเพิ่ม (Extra work)</t>
@@ -1357,7 +1466,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ขึ้นการ์ดสรุป "ตัด Slab จาก Block": Block เหลือ 6.18 CBM, ขนาดเป้าหมาย 2.75 × 1.45, Polished หนา 0.02, ประมาณ 77 แผ่น / 307.04 ตร.ม., ผูกกับ งานเพิ่ม และข้อความสีเขียว "แผนใช้ 6.14 CBM พอ" (ตัวอย่างจริง EG01/STCUT/00047)</t>
+          <t>ขึ้นการ์ดสรุป "ตัด Slab จาก Block": Block เหลือ 6.18 CBM, ขนาดเป้าหมาย 2.75 × 1.45, Polished หนา 0.02, ประมาณ 65 แผ่น / 259.19 ตร.ม., ผูกกับ งานเพิ่ม และข้อความสีเขียว "แผนใช้ 6.10 CBM (รวมสูญเสียเลื่อย 15%) พอ" (ตัวอย่างจริง EG01/STCUT/00214)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1367,7 +1476,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>จำนวนแผ่นที่ระบบคำนวณเป็นค่าสูงสุดตามทฤษฎี (ความกว้างก้อน ÷ ความหนา) ไม่หักเนื้อหินที่หายไปกับใบเลื่อย ของจริงอาจได้น้อยกว่า (รอตกลงกับลูกค้า) · ใบตัดไม่มี SO ต้องเลือกเหตุผลก่อน Confirm</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — จำนวนแผ่นและ CBM ที่ใช้หัก "% สูญเสียจากการเลื่อย" แล้ว (ค่าเริ่มต้นบริษัท 15% ปรับเป็นรายก้อนได้) จึงได้ 65 แผ่น ไม่ใช่ 77 แผ่นเหมือนรอบก่อน
+ข้อความสีเขียวบอกว่า "แผนใช้ 6.10 CBM (รวมสูญเสียเลื่อย 15%) พอ" · ใบตัดไม่มี SO ต้องเลือกเหตุผลก่อน Confirm</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1395,7 +1505,7 @@
         <is>
           <t>1. กดปุ่ม ย้ายไปสถานีตัด (ระบบย้าย Block จากคลังไป Stone Production)
 2. รีเฟรชหน้า แล้วกด Confirm
-3. กด Complete Cut และยืนยันตามหน้าต่างที่ขึ้น</t>
+3. กด ตัดเสร็จ (Complete Cut)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1405,7 +1515,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบตัดเป็น Done — ตัดได้จริง 77 แผ่น / 307.04 ตร.ม. (100% ของแผน), Block ใช้ 6.14 ลบ.ม. เหลือ 0.04 ลบ.ม., ได้ Lot ของแผ่น 77 ใบ (ปุ่ม Serial Numbers ขึ้น 77) อยู่ใน Stone Available</t>
+          <t>ใบตัดเป็น Done — ตัดได้จริง 65 แผ่น / 259.19 ตร.ม. (100% ของแผน), Block ใช้ 6.10 ลบ.ม. เหลือ 0.08 ลบ.ม., ได้ Lot ของแผ่น 65 ใบ (ปุ่ม Serial Numbers ขึ้น 65) อยู่ใน Stone Available · มูลค่าที่ย้ายจาก Block เป็น Slab 164,838.19 บาท (แผ่นละ 2,535.97)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1415,7 +1525,8 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>หลังกด ย้ายไปสถานีตัด แถบเหลืองเตือนอาจยังค้างอยู่ ให้รีเฟรชหน้า (บั๊กการแสดงผลที่จดไว้ ข้อมูลถูกต้อง)</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ต้นทุนแผ่นแบ่งตามต้นทุนของ Block ก้อนนั้นเอง (ตันตามใบส่งของ × ราคาต่อตัน) ตามปริมาตรที่ใช้จริง รวมส่วนที่เสียไปกับใบเลื่อย
+หลังกด ย้ายไปสถานีตัด ให้รีเฟรชหน้าแล้วกด Confirm · ปุ่ม Complete Cut ชื่อ "ตัดเสร็จ"</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -1437,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1457,7 +1568,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F. คืน Block ให้ผู้ขาย — ใบคืนจองก้อนเดิมให้เอง และเลือกก้อนอื่นไม่ได้</t>
+          <t>F. คืน Block ให้ผู้ขาย — ใบคืนจองก้อนเดิมให้เอง</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1647,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มี PO และใบรับของที่ Done ของ Block 1 ก้อนที่ยังไม่ถูกตัด (ทดสอบด้วย PO แยกต่างหาก ไม่ใช่ P00086)</t>
+          <t>มี PO และใบรับของที่ Done ของ Block 1 ก้อนที่ยังไม่ถูกตัด และมีบิลผู้ขายที่ Posted (ทดสอบด้วย PO แยกต่างหาก ไม่ใช่ P00295)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1549,13 +1660,14 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>PO ทดสอบ = P00090 (Qty (Ton) 5.40 = 2.00 ลบ.ม. @ 27,000 ต่อ ลบ.ม.)
-Block = 2.00 × 1.00 × 1.00 ม. (BLK-26-0034)</t>
+          <t>PO ทดสอบ = P00296 (2.00 ลบ.ม. @ 27,000 ต่อ ลบ.ม.)
+Block = 2.00 × 1.00 × 1.00 ม. · ตันตามใบส่งของ 5.500 (BLK-26-0387)
+บิลผู้ขาย = BILL/2026/10/0007 (5.500 ตัน × 10,000 = 55,000)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบคืน Done Quantity 2.00 ลบ.ม. (5.40 ตัน) · ช่อง Received ของ PO กลับเป็น 0.00 · เอกสาร Block ยังอยู่เป็นประวัติ ขึ้นป้าย "ใช้หมดแล้ว" คงเหลือ 0.00 CBM (ตัวอย่างจริง EG01/OUT/00102)</t>
+          <t>ใบคืน Done Quantity 2.00 ลบ.ม. · มูลค่าสต็อกที่ตัดออก 55,000.00 (เท่าตอนรับ) · ช่อง Received ของ PO กลับเป็น 0.00 · เอกสาร Block ยังอยู่เป็นประวัติ ขึ้นป้าย "ใช้หมดแล้ว" คงเหลือ 0.00 CBM (ตัวอย่างจริง EG01/IN/00361 → ใบคืน EG01/OUT/00320)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1565,13 +1677,63 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>✅ แก้แล้ว 11 ต.ค. 2569: ใบคืน Block ขึ้น Ready พร้อมก้อนเดิมให้เองและเลือกได้เฉพาะก้อนของใบรับของเดิม (ก่อนแก้ใบคืนค้าง Waiting ต้องเลือกก้อนและกรอกขนาดเอง) · คืนได้เฉพาะ Block ที่ยังไม่ถูกตัด Block ที่ตัดบางส่วนแล้วยังไม่ได้ทดลอง</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ใบคืนตีมูลค่าเท่าใบรับของเดิมของก้อนนั้น (55,000 ตามตัน 5.50 × 10,000) ไม่ใช่ราคา FIFO ชั้นเก่าสุด · ตัวอย่างนี้สร้างบิลผู้ขายไว้ก่อนคืนเพื่อใช้ต่อใน TC-GP-BPC-14
+ใบคืน Block ขึ้น Ready พร้อมก้อนเดิมให้เองและเลือกได้เฉพาะก้อนของใบรับของเดิม · คืนได้เฉพาะ Block ที่ยังไม่ถูกตัด · คอลัมน์ Qty (Ton) บนใบคืนแสดง 5.40 (คำนวณจาก CBM) ต่างจากตันตามใบส่งของ 5.50 แต่มูลค่าและใบลดหนี้ใช้ 5.50</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
       <c r="L4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-BPC-14</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>ออกใบลดหนี้ผู้ขายหลังคืน Block (เป็นตัน)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-BPC-08 เสร็จแล้ว (มีบิลผู้ขาย BILL/2026/10/0007 และใบคืนที่ Done)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดบิลผู้ขายของ PO ที่คืน (BILL/2026/10/0007)
+2. กดปุ่ม Credit Note แล้วกด Reverse ในหน้าต่าง
+3. ตรวจบรรทัดสินค้าในใบลดหนี้ แล้วกด Confirm</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>ใบลดหนี้ผู้ขาย RBILL/2026/10/0001: Qty (Ton) 5.50 · Quantity 5.500 ตัน · Price / Ton 10,000.00 · Amount 55,000.00 · VAT 7% 3,850.00 · Total 58,850.00 บาท สถานะ Posted ขึ้นป้าย PAID Amount Due 0.00</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ใบลดหนี้ของ Block เขียนเป็นตัน ตรงกับบิลเดิม (Quantity 5.500 ตัน ไม่แปลงเป็น ลบ.ม.) จึงตัดยอดบิลได้พอดี
+ใบลดหนี้ที่สร้างจากบิลเดิมด้วยปุ่ม Credit Note ถูกจับคู่กับบิลเดิมให้เอง ยอดคงค้างเป็น 0</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1686,27 +1848,27 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-BPC-05 เสร็จแล้ว (BLK-26-0029 แก้ขนาดเป็น 6.73 ลบ.ม.) และยังไม่ถูกขายหรือตัด · มีลูกค้าในระบบ</t>
+          <t>ทำ TC-GP-BPC-05 เสร็จแล้ว (BLK-26-0385 แก้ขนาดเป็น 6.73 ลบ.ม.) และยังไม่ถูกขายหรือตัด · มีลูกค้าในระบบ</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิดแอป Sales &gt; Orders &gt; Quotations &gt; New
-2. เลือก Customer แล้วกด "Add a product" เลือก "SHANDONG BLACK - Block"
-3. กดปุ่ม "Sell Whole Block" ที่บรรทัดสินค้า แล้วเลือก BLK-26-0029
+2. เลือก Customer แล้วกด "Add a product" เลือก "SHANDONG BLACK - Block" แล้วกด Save
+3. กดปุ่ม "Sell Whole Block" ที่บรรทัดสินค้า แล้วเลือก BLK-26-0385
 4. ใส่ราคาต่อ ลบ.ม. ตรวจจำนวนและยอดรวม แล้วกด Confirm</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Customer = Demo Hotel Customer
-Block = BLK-26-0029
+Block = BLK-26-0385
 Unit Price = 70,200 บาท ต่อ ลบ.ม.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดขายขึ้น Qty (Ton) 18.17, Quantity 6.73 ลบ.ม., ราคา 70,200 · ยอดก่อน VAT 472,446.00, VAT 7% 33,071.22 บาท · หลัง Confirm เป็น Sales Order และมีปุ่มสมาร์ท Delivery 1 ใบ (ตัวอย่างจริง S00209)</t>
+          <t>บรรทัดขายขึ้น Qty (Ton) 18.17, Quantity 6.73 ลบ.ม., ราคา 70,200 · ยอดก่อน VAT 472,446.00, VAT 7% 33,071.22 บาท · หลัง Confirm เป็น Sales Order และมีปุ่มสมาร์ท Delivery 1 ใบ (ตัวอย่างจริง S00616)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1716,7 +1878,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Block ขายเป็นลูกบาศก์เมตร ช่อง Qty (Ton) อยู่หน้า Quantity ให้ดูน้ำหนักประกอบ · ขายสินค้า Block (ลงท้าย - Block) ไม่ใช่สินค้า FG · ขนาดที่ขายคือขนาดล่าสุดของก้อน (หลังแก้ขนาดแล้ว)</t>
+          <t>Block ขายเป็นลูกบาศก์เมตร ช่อง Qty (Ton) อยู่หน้า Quantity ให้ดูน้ำหนักประกอบ (18.17 คำนวณจาก CBM ใหม่ ต่างจากตันของ Block 18.80 ซึ่งใช้คิดต้นทุน) · ขายสินค้า Block (ลงท้าย - Block) ไม่ใช่สินค้า FG · ขนาดที่ขายคือขนาดล่าสุดของก้อน (หลังแก้ขนาดแล้ว) · คอลัมน์เสริม (ขนาด/ราคา, หนา, เตือนกำไร, Slabs) ถูกซ่อนในภาพ</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1754,7 +1916,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของ Done — Source Location Stone Inventory/Stone Available, Demand 6.73 = Quantity 6.73 ลบ.ม., Qty (Ton) 18.17 · BLK-26-0029 คงเหลือ 0.00 ลบ.ม. (ตัวอย่างจริง EG01/OUT/00103)</t>
+          <t>ใบส่งของ Done — Source Location Stone Inventory/Stone Available, Demand 6.73 = Quantity 6.73 ลบ.ม., Qty (Ton) 18.17 · BLK-26-0385 คงเหลือ 0.00 ลบ.ม. (ตัวอย่างจริง EG01/OUT/00321)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1802,7 +1964,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ Posted ยอดก่อน VAT 472,446.00, VAT 33,071.22, รวม 505,517.22 · Journal Items: Credit 411100 รายได้ 472,446.00, Credit 113120 สต็อก 181,710.00 คู่กับ Debit 511110 ต้นทุนขาย 181,710.00, Credit 213200 VAT 33,071.22 (ตัวอย่างจริง INV/2026/00020)</t>
+          <t>ใบแจ้งหนี้ Posted ยอดก่อน VAT 472,446.00, VAT 33,071.22, รวม 505,517.22 · Journal Items: Credit 411100 รายได้ 472,446.00, Credit 113120 สต็อก 181,787.36 คู่กับ Debit 511110 ต้นทุนขาย 181,787.36, Credit 213200 VAT 33,071.22 (ตัวอย่างจริง INV/2026/00030)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1812,7 +1974,8 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>ต้นทุนขายมาจากราคาซื้อจริง 27,000 × 6.73 = 181,710 (ไม่ใช่ราคาขาย) · ฝ่ายบัญชีตรวจได้จากแท็บ Journal Items</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ต้นทุนขายคือต้นทุนของ Block ก้อนนั้นเอง (ซื้อ 18.80 ตัน × 10,000 = 188,000 หักส่วนที่ปรับลดตอนแก้ขนาด) ไม่ใช่ชั้น FIFO เก่าสุดหรือ ตัน × 10,000 ที่คำนวณใหม่
+ต้นทุนขาย 181,787.36 มาจากราคาซื้อจริงของก้อนนี้ (ไม่ใช่ราคาขาย) · ฝ่ายบัญชีตรวจได้จากแท็บ Journal Items · ส่วนต่างจาก 188,000 คือ 6,212.64 จากการปรับสต็อก -0.23 ลบ.ม. ตอนแก้ขนาด (TC-GP-BPC-05)</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>

</xml_diff>